<commit_message>
Create GUS gas master Excel for 2018
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -511,7 +511,7 @@
         <v>2018</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>2</v>
@@ -538,7 +538,7 @@
         <v>2018</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>1</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:R3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -581,6 +581,7 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -611,60 +612,65 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>2018 M01</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2018 M02</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2018 M03</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2018 M04</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2018 M05</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2018 M06</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>2018 M07</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2018 M08</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>2018 M09</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>2018 M10</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>2018 M11</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>2018 M12</t>
         </is>
@@ -697,39 +703,42 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
+        <v>107182</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>5087</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>4949</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>9924</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>10053</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>8551</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>13587</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>10231</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>9890</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>4951</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="P2" s="3" t="n">
         <v>9915</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>8443</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="R2" s="3" t="n">
         <v>11601</v>
       </c>
     </row>
@@ -760,39 +769,42 @@
         </is>
       </c>
       <c r="F3" s="3" t="n">
+        <v>498884</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>46688</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>45438</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>57736</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>33793</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="K3" s="3" t="n">
         <v>40487</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>40126</v>
       </c>
-      <c r="L3" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>38068</v>
       </c>
-      <c r="M3" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>39250</v>
       </c>
-      <c r="N3" s="3" t="n">
+      <c r="O3" s="3" t="n">
         <v>43116</v>
       </c>
-      <c r="O3" s="3" t="n">
+      <c r="P3" s="3" t="n">
         <v>35482</v>
       </c>
-      <c r="P3" s="3" t="n">
+      <c r="Q3" s="3" t="n">
         <v>36555</v>
       </c>
-      <c r="Q3" s="3" t="n">
+      <c r="R3" s="3" t="n">
         <v>42145</v>
       </c>
     </row>
@@ -807,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:R2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -827,6 +839,7 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -857,60 +870,65 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
+          <t>2018</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
           <t>2018 M01</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>2018 M02</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>2018 M03</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>2018 M04</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>2018 M05</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>2018 M06</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>2018 M07</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>2018 M08</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>2018 M09</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>2018 M10</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>2018 M11</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>2018 M12</t>
         </is>
@@ -943,39 +961,42 @@
         </is>
       </c>
       <c r="F2" s="3" t="n">
+        <v>27715</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>4003</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>2049</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>2752</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>3114</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>1476</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>1557</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="M2" s="3" t="n">
         <v>3107</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="N2" s="3" t="n">
         <v>3247</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="O2" s="3" t="n">
         <v>732</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="P2" s="3" t="n">
         <v>2363</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>2070</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="R2" s="3" t="n">
         <v>1245</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Append GUS gas data for 2019
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2018</v>
+        <v>2019</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>13</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R3"/>
+  <dimension ref="A1:AE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -582,6 +582,19 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -675,6 +688,71 @@
           <t>2018 M12</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M01</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M02</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M03</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M04</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M05</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M06</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M07</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M08</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M09</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M10</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M11</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -741,6 +819,45 @@
       <c r="R2" s="3" t="n">
         <v>11601</v>
       </c>
+      <c r="S2" s="3" t="n">
+        <v>135294</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>11852</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>8476</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>8376</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>12398</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>15174</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>13677</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>9060</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>10064</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>8753</v>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>9900</v>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v>13755</v>
+      </c>
+      <c r="AE2" s="3" t="n">
+        <v>13809</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -806,6 +923,45 @@
       </c>
       <c r="R3" s="3" t="n">
         <v>42145</v>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>537428</v>
+      </c>
+      <c r="T3" s="3" t="n">
+        <v>50582</v>
+      </c>
+      <c r="U3" s="3" t="n">
+        <v>44805</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>49565</v>
+      </c>
+      <c r="W3" s="3" t="n">
+        <v>45537</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>48084</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>36830</v>
+      </c>
+      <c r="Z3" s="3" t="n">
+        <v>45286</v>
+      </c>
+      <c r="AA3" s="3" t="n">
+        <v>39268</v>
+      </c>
+      <c r="AB3" s="3" t="n">
+        <v>44997</v>
+      </c>
+      <c r="AC3" s="3" t="n">
+        <v>44025</v>
+      </c>
+      <c r="AD3" s="3" t="n">
+        <v>43628</v>
+      </c>
+      <c r="AE3" s="3" t="n">
+        <v>44821</v>
       </c>
     </row>
   </sheetData>
@@ -819,7 +975,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R2"/>
+  <dimension ref="A1:AE2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -840,6 +996,19 @@
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="10" customWidth="1" min="19" max="19"/>
+    <col width="10" customWidth="1" min="20" max="20"/>
+    <col width="10" customWidth="1" min="21" max="21"/>
+    <col width="10" customWidth="1" min="22" max="22"/>
+    <col width="10" customWidth="1" min="23" max="23"/>
+    <col width="10" customWidth="1" min="24" max="24"/>
+    <col width="10" customWidth="1" min="25" max="25"/>
+    <col width="10" customWidth="1" min="26" max="26"/>
+    <col width="10" customWidth="1" min="27" max="27"/>
+    <col width="10" customWidth="1" min="28" max="28"/>
+    <col width="10" customWidth="1" min="29" max="29"/>
+    <col width="10" customWidth="1" min="30" max="30"/>
+    <col width="10" customWidth="1" min="31" max="31"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -933,6 +1102,71 @@
           <t>2018 M12</t>
         </is>
       </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M01</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M02</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M03</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M04</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M05</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M06</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M07</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M08</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M09</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M10</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M11</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>2019 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -998,6 +1232,45 @@
       </c>
       <c r="R2" s="3" t="n">
         <v>1245</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>26578</v>
+      </c>
+      <c r="T2" s="3" t="n">
+        <v>1538</v>
+      </c>
+      <c r="U2" s="3" t="n">
+        <v>3492</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>5898</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>2348</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>161</v>
+      </c>
+      <c r="Y2" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="Z2" s="3" t="n">
+        <v>421</v>
+      </c>
+      <c r="AA2" s="3" t="n">
+        <v>429</v>
+      </c>
+      <c r="AB2" s="3" t="n">
+        <v>1232</v>
+      </c>
+      <c r="AC2" s="3" t="n">
+        <v>6991</v>
+      </c>
+      <c r="AD2" s="3" t="n">
+        <v>2683</v>
+      </c>
+      <c r="AE2" s="3" t="n">
+        <v>1223</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2020
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,13 +535,13 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2019</v>
+        <v>2020</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>13</v>
+        <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F3" s="3" t="b">
         <v>1</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE3"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -595,6 +595,19 @@
     <col width="10" customWidth="1" min="29" max="29"/>
     <col width="10" customWidth="1" min="30" max="30"/>
     <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
+    <col width="10" customWidth="1" min="33" max="33"/>
+    <col width="10" customWidth="1" min="34" max="34"/>
+    <col width="10" customWidth="1" min="35" max="35"/>
+    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="10" customWidth="1" min="37" max="37"/>
+    <col width="10" customWidth="1" min="38" max="38"/>
+    <col width="10" customWidth="1" min="39" max="39"/>
+    <col width="10" customWidth="1" min="40" max="40"/>
+    <col width="10" customWidth="1" min="41" max="41"/>
+    <col width="10" customWidth="1" min="42" max="42"/>
+    <col width="10" customWidth="1" min="43" max="43"/>
+    <col width="10" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -753,6 +766,71 @@
           <t>2019 M12</t>
         </is>
       </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M01</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M02</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M03</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M04</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M05</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M06</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M07</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M08</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M09</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M10</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M11</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -858,6 +936,45 @@
       <c r="AE2" s="3" t="n">
         <v>13809</v>
       </c>
+      <c r="AF2" s="3" t="n">
+        <v>150899</v>
+      </c>
+      <c r="AG2" s="3" t="n">
+        <v>15508</v>
+      </c>
+      <c r="AH2" s="3" t="n">
+        <v>12326</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>11566</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>17926</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>16743</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>13555</v>
+      </c>
+      <c r="AM2" s="3" t="n">
+        <v>8240</v>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v>11937</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>10327</v>
+      </c>
+      <c r="AP2" s="3" t="n">
+        <v>8399</v>
+      </c>
+      <c r="AQ2" s="3" t="n">
+        <v>15317</v>
+      </c>
+      <c r="AR2" s="3" t="n">
+        <v>9055</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -962,6 +1079,45 @@
       </c>
       <c r="AE3" s="3" t="n">
         <v>44821</v>
+      </c>
+      <c r="AF3" s="3" t="n">
+        <v>519548</v>
+      </c>
+      <c r="AG3" s="3" t="n">
+        <v>29575</v>
+      </c>
+      <c r="AH3" s="3" t="n">
+        <v>36582</v>
+      </c>
+      <c r="AI3" s="3" t="n">
+        <v>51589</v>
+      </c>
+      <c r="AJ3" s="3" t="n">
+        <v>41604</v>
+      </c>
+      <c r="AK3" s="3" t="n">
+        <v>45584</v>
+      </c>
+      <c r="AL3" s="3" t="n">
+        <v>43893</v>
+      </c>
+      <c r="AM3" s="3" t="n">
+        <v>53194</v>
+      </c>
+      <c r="AN3" s="3" t="n">
+        <v>49247</v>
+      </c>
+      <c r="AO3" s="3" t="n">
+        <v>36175</v>
+      </c>
+      <c r="AP3" s="3" t="n">
+        <v>43502</v>
+      </c>
+      <c r="AQ3" s="3" t="n">
+        <v>42222</v>
+      </c>
+      <c r="AR3" s="3" t="n">
+        <v>46381</v>
       </c>
     </row>
   </sheetData>
@@ -975,7 +1131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AE2"/>
+  <dimension ref="A1:AR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1009,6 +1165,19 @@
     <col width="10" customWidth="1" min="29" max="29"/>
     <col width="10" customWidth="1" min="30" max="30"/>
     <col width="10" customWidth="1" min="31" max="31"/>
+    <col width="10" customWidth="1" min="32" max="32"/>
+    <col width="10" customWidth="1" min="33" max="33"/>
+    <col width="10" customWidth="1" min="34" max="34"/>
+    <col width="10" customWidth="1" min="35" max="35"/>
+    <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="10" customWidth="1" min="37" max="37"/>
+    <col width="10" customWidth="1" min="38" max="38"/>
+    <col width="10" customWidth="1" min="39" max="39"/>
+    <col width="10" customWidth="1" min="40" max="40"/>
+    <col width="10" customWidth="1" min="41" max="41"/>
+    <col width="10" customWidth="1" min="42" max="42"/>
+    <col width="10" customWidth="1" min="43" max="43"/>
+    <col width="10" customWidth="1" min="44" max="44"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1167,6 +1336,71 @@
           <t>2019 M12</t>
         </is>
       </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M01</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M02</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M03</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M04</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M05</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M06</t>
+        </is>
+      </c>
+      <c r="AM1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M07</t>
+        </is>
+      </c>
+      <c r="AN1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M08</t>
+        </is>
+      </c>
+      <c r="AO1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M09</t>
+        </is>
+      </c>
+      <c r="AP1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M10</t>
+        </is>
+      </c>
+      <c r="AQ1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M11</t>
+        </is>
+      </c>
+      <c r="AR1" s="1" t="inlineStr">
+        <is>
+          <t>2020 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1186,91 +1420,222 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>27111100 - Gaz ziemny skroplony [TJ]</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>POLSKA</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="3" t="n">
+        <v>718</v>
+      </c>
+      <c r="AG2" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="AH2" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="AI2" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="AJ2" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="AK2" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="AL2" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="AM2" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="AN2" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="AO2" s="3" t="n">
+        <v>73</v>
+      </c>
+      <c r="AP2" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="AQ2" s="3" t="n">
+        <v>72</v>
+      </c>
+      <c r="AR2" s="3" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Eksport towarów</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>[-]</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Ogółem</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
           <t>27112100 - Gaz ziemny w stanie gazowym [TJ]</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="E3" s="2" t="inlineStr">
         <is>
           <t>POLSKA</t>
         </is>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="F3" s="3" t="n">
         <v>27715</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="G3" s="3" t="n">
         <v>4003</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="H3" s="3" t="n">
         <v>2049</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="I3" s="3" t="n">
         <v>2752</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="J3" s="3" t="n">
         <v>3114</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="K3" s="3" t="n">
         <v>1476</v>
       </c>
-      <c r="L2" s="3" t="n">
+      <c r="L3" s="3" t="n">
         <v>1557</v>
       </c>
-      <c r="M2" s="3" t="n">
+      <c r="M3" s="3" t="n">
         <v>3107</v>
       </c>
-      <c r="N2" s="3" t="n">
+      <c r="N3" s="3" t="n">
         <v>3247</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="O3" s="3" t="n">
         <v>732</v>
       </c>
-      <c r="P2" s="3" t="n">
+      <c r="P3" s="3" t="n">
         <v>2363</v>
       </c>
-      <c r="Q2" s="3" t="n">
+      <c r="Q3" s="3" t="n">
         <v>2070</v>
       </c>
-      <c r="R2" s="3" t="n">
+      <c r="R3" s="3" t="n">
         <v>1245</v>
       </c>
-      <c r="S2" s="3" t="n">
+      <c r="S3" s="3" t="n">
         <v>26578</v>
       </c>
-      <c r="T2" s="3" t="n">
+      <c r="T3" s="3" t="n">
         <v>1538</v>
       </c>
-      <c r="U2" s="3" t="n">
+      <c r="U3" s="3" t="n">
         <v>3492</v>
       </c>
-      <c r="V2" s="3" t="n">
+      <c r="V3" s="3" t="n">
         <v>5898</v>
       </c>
-      <c r="W2" s="3" t="n">
+      <c r="W3" s="3" t="n">
         <v>2348</v>
       </c>
-      <c r="X2" s="3" t="n">
+      <c r="X3" s="3" t="n">
         <v>161</v>
       </c>
-      <c r="Y2" s="3" t="n">
+      <c r="Y3" s="3" t="n">
         <v>162</v>
       </c>
-      <c r="Z2" s="3" t="n">
+      <c r="Z3" s="3" t="n">
         <v>421</v>
       </c>
-      <c r="AA2" s="3" t="n">
+      <c r="AA3" s="3" t="n">
         <v>429</v>
       </c>
-      <c r="AB2" s="3" t="n">
+      <c r="AB3" s="3" t="n">
         <v>1232</v>
       </c>
-      <c r="AC2" s="3" t="n">
+      <c r="AC3" s="3" t="n">
         <v>6991</v>
       </c>
-      <c r="AD2" s="3" t="n">
+      <c r="AD3" s="3" t="n">
         <v>2683</v>
       </c>
-      <c r="AE2" s="3" t="n">
+      <c r="AE3" s="3" t="n">
         <v>1223</v>
+      </c>
+      <c r="AF3" s="3" t="n">
+        <v>38359</v>
+      </c>
+      <c r="AG3" s="3" t="n">
+        <v>2588</v>
+      </c>
+      <c r="AH3" s="3" t="n">
+        <v>5849</v>
+      </c>
+      <c r="AI3" s="3" t="n">
+        <v>4918</v>
+      </c>
+      <c r="AJ3" s="3" t="n">
+        <v>5702</v>
+      </c>
+      <c r="AK3" s="3" t="n">
+        <v>6626</v>
+      </c>
+      <c r="AL3" s="3" t="n">
+        <v>2844</v>
+      </c>
+      <c r="AM3" s="3" t="n">
+        <v>3649</v>
+      </c>
+      <c r="AN3" s="3" t="n">
+        <v>3273</v>
+      </c>
+      <c r="AO3" s="3" t="n">
+        <v>2009</v>
+      </c>
+      <c r="AP3" s="3" t="n">
+        <v>887</v>
+      </c>
+      <c r="AQ3" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="AR3" s="3" t="n">
+        <v>2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2021
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2020</v>
+        <v>2021</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>2</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:BE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -608,6 +608,19 @@
     <col width="10" customWidth="1" min="42" max="42"/>
     <col width="10" customWidth="1" min="43" max="43"/>
     <col width="10" customWidth="1" min="44" max="44"/>
+    <col width="10" customWidth="1" min="45" max="45"/>
+    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="10" customWidth="1" min="47" max="47"/>
+    <col width="10" customWidth="1" min="48" max="48"/>
+    <col width="10" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="10" customWidth="1" min="51" max="51"/>
+    <col width="10" customWidth="1" min="52" max="52"/>
+    <col width="10" customWidth="1" min="53" max="53"/>
+    <col width="10" customWidth="1" min="54" max="54"/>
+    <col width="10" customWidth="1" min="55" max="55"/>
+    <col width="10" customWidth="1" min="56" max="56"/>
+    <col width="10" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -831,6 +844,71 @@
           <t>2020 M12</t>
         </is>
       </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M01</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M02</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M03</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M04</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M05</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M06</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M07</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M08</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M09</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M10</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M11</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -975,6 +1053,45 @@
       <c r="AR2" s="3" t="n">
         <v>9055</v>
       </c>
+      <c r="AS2" s="3" t="n">
+        <v>159182</v>
+      </c>
+      <c r="AT2" s="3" t="n">
+        <v>8937</v>
+      </c>
+      <c r="AU2" s="3" t="n">
+        <v>9308</v>
+      </c>
+      <c r="AV2" s="3" t="n">
+        <v>13993</v>
+      </c>
+      <c r="AW2" s="3" t="n">
+        <v>18996</v>
+      </c>
+      <c r="AX2" s="3" t="n">
+        <v>16812</v>
+      </c>
+      <c r="AY2" s="3" t="n">
+        <v>14095</v>
+      </c>
+      <c r="AZ2" s="3" t="n">
+        <v>16109</v>
+      </c>
+      <c r="BA2" s="3" t="n">
+        <v>9083</v>
+      </c>
+      <c r="BB2" s="3" t="n">
+        <v>10393</v>
+      </c>
+      <c r="BC2" s="3" t="n">
+        <v>5497</v>
+      </c>
+      <c r="BD2" s="3" t="n">
+        <v>17754</v>
+      </c>
+      <c r="BE2" s="3" t="n">
+        <v>18205</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1118,6 +1235,45 @@
       </c>
       <c r="AR3" s="3" t="n">
         <v>46381</v>
+      </c>
+      <c r="AS3" s="3" t="n">
+        <v>553844</v>
+      </c>
+      <c r="AT3" s="3" t="n">
+        <v>54864</v>
+      </c>
+      <c r="AU3" s="3" t="n">
+        <v>53922</v>
+      </c>
+      <c r="AV3" s="3" t="n">
+        <v>46215</v>
+      </c>
+      <c r="AW3" s="3" t="n">
+        <v>47184</v>
+      </c>
+      <c r="AX3" s="3" t="n">
+        <v>32884</v>
+      </c>
+      <c r="AY3" s="3" t="n">
+        <v>51328</v>
+      </c>
+      <c r="AZ3" s="3" t="n">
+        <v>42825</v>
+      </c>
+      <c r="BA3" s="3" t="n">
+        <v>43369</v>
+      </c>
+      <c r="BB3" s="3" t="n">
+        <v>39706</v>
+      </c>
+      <c r="BC3" s="3" t="n">
+        <v>44913</v>
+      </c>
+      <c r="BD3" s="3" t="n">
+        <v>45352</v>
+      </c>
+      <c r="BE3" s="3" t="n">
+        <v>51282</v>
       </c>
     </row>
   </sheetData>
@@ -1131,7 +1287,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR3"/>
+  <dimension ref="A1:BE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1178,6 +1334,19 @@
     <col width="10" customWidth="1" min="42" max="42"/>
     <col width="10" customWidth="1" min="43" max="43"/>
     <col width="10" customWidth="1" min="44" max="44"/>
+    <col width="10" customWidth="1" min="45" max="45"/>
+    <col width="10" customWidth="1" min="46" max="46"/>
+    <col width="10" customWidth="1" min="47" max="47"/>
+    <col width="10" customWidth="1" min="48" max="48"/>
+    <col width="10" customWidth="1" min="49" max="49"/>
+    <col width="10" customWidth="1" min="50" max="50"/>
+    <col width="10" customWidth="1" min="51" max="51"/>
+    <col width="10" customWidth="1" min="52" max="52"/>
+    <col width="10" customWidth="1" min="53" max="53"/>
+    <col width="10" customWidth="1" min="54" max="54"/>
+    <col width="10" customWidth="1" min="55" max="55"/>
+    <col width="10" customWidth="1" min="56" max="56"/>
+    <col width="10" customWidth="1" min="57" max="57"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1399,6 +1568,71 @@
       <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>2020 M12</t>
+        </is>
+      </c>
+      <c r="AS1" s="1" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="AT1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M01</t>
+        </is>
+      </c>
+      <c r="AU1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M02</t>
+        </is>
+      </c>
+      <c r="AV1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M03</t>
+        </is>
+      </c>
+      <c r="AW1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M04</t>
+        </is>
+      </c>
+      <c r="AX1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M05</t>
+        </is>
+      </c>
+      <c r="AY1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M06</t>
+        </is>
+      </c>
+      <c r="AZ1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M07</t>
+        </is>
+      </c>
+      <c r="BA1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M08</t>
+        </is>
+      </c>
+      <c r="BB1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M09</t>
+        </is>
+      </c>
+      <c r="BC1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M10</t>
+        </is>
+      </c>
+      <c r="BD1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M11</t>
+        </is>
+      </c>
+      <c r="BE1" s="1" t="inlineStr">
+        <is>
+          <t>2021 M12</t>
         </is>
       </c>
     </row>
@@ -1493,6 +1727,45 @@
       <c r="AR2" s="3" t="n">
         <v>72</v>
       </c>
+      <c r="AS2" s="3" t="n">
+        <v>1419</v>
+      </c>
+      <c r="AT2" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="AU2" s="3" t="n">
+        <v>88</v>
+      </c>
+      <c r="AV2" s="3" t="n">
+        <v>108</v>
+      </c>
+      <c r="AW2" s="3" t="n">
+        <v>112</v>
+      </c>
+      <c r="AX2" s="3" t="n">
+        <v>133</v>
+      </c>
+      <c r="AY2" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="AZ2" s="3" t="n">
+        <v>186</v>
+      </c>
+      <c r="BA2" s="3" t="n">
+        <v>107</v>
+      </c>
+      <c r="BB2" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="BC2" s="3" t="n">
+        <v>95</v>
+      </c>
+      <c r="BD2" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="BE2" s="3" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1636,6 +1909,39 @@
       </c>
       <c r="AR3" s="3" t="n">
         <v>2</v>
+      </c>
+      <c r="AS3" s="3" t="n">
+        <v>2979</v>
+      </c>
+      <c r="AT3" s="2" t="inlineStr"/>
+      <c r="AU3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AV3" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="AW3" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="AX3" s="2" t="inlineStr"/>
+      <c r="AY3" s="2" t="inlineStr"/>
+      <c r="AZ3" s="3" t="n">
+        <v>271</v>
+      </c>
+      <c r="BA3" s="3" t="n">
+        <v>1312</v>
+      </c>
+      <c r="BB3" s="3" t="n">
+        <v>1037</v>
+      </c>
+      <c r="BC3" s="3" t="n">
+        <v>67</v>
+      </c>
+      <c r="BD3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="BE3" s="3" t="n">
+        <v>279</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2022
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2021</v>
+        <v>2022</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>2</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE3"/>
+  <dimension ref="A1:BR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -621,6 +621,19 @@
     <col width="10" customWidth="1" min="55" max="55"/>
     <col width="10" customWidth="1" min="56" max="56"/>
     <col width="10" customWidth="1" min="57" max="57"/>
+    <col width="10" customWidth="1" min="58" max="58"/>
+    <col width="10" customWidth="1" min="59" max="59"/>
+    <col width="10" customWidth="1" min="60" max="60"/>
+    <col width="10" customWidth="1" min="61" max="61"/>
+    <col width="10" customWidth="1" min="62" max="62"/>
+    <col width="10" customWidth="1" min="63" max="63"/>
+    <col width="10" customWidth="1" min="64" max="64"/>
+    <col width="10" customWidth="1" min="65" max="65"/>
+    <col width="10" customWidth="1" min="66" max="66"/>
+    <col width="10" customWidth="1" min="67" max="67"/>
+    <col width="10" customWidth="1" min="68" max="68"/>
+    <col width="10" customWidth="1" min="69" max="69"/>
+    <col width="10" customWidth="1" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -909,6 +922,71 @@
           <t>2021 M12</t>
         </is>
       </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M01</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M02</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M03</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M04</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M05</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M06</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M07</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M08</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M09</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M10</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M11</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1092,6 +1170,45 @@
       <c r="BE2" s="3" t="n">
         <v>18205</v>
       </c>
+      <c r="BF2" s="3" t="n">
+        <v>242932</v>
+      </c>
+      <c r="BG2" s="3" t="n">
+        <v>9044</v>
+      </c>
+      <c r="BH2" s="3" t="n">
+        <v>13427</v>
+      </c>
+      <c r="BI2" s="3" t="n">
+        <v>20940</v>
+      </c>
+      <c r="BJ2" s="3" t="n">
+        <v>17438</v>
+      </c>
+      <c r="BK2" s="3" t="n">
+        <v>24679</v>
+      </c>
+      <c r="BL2" s="3" t="n">
+        <v>23846</v>
+      </c>
+      <c r="BM2" s="3" t="n">
+        <v>25119</v>
+      </c>
+      <c r="BN2" s="3" t="n">
+        <v>16158</v>
+      </c>
+      <c r="BO2" s="3" t="n">
+        <v>17259</v>
+      </c>
+      <c r="BP2" s="3" t="n">
+        <v>25273</v>
+      </c>
+      <c r="BQ2" s="3" t="n">
+        <v>21481</v>
+      </c>
+      <c r="BR2" s="3" t="n">
+        <v>28268</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1274,6 +1391,45 @@
       </c>
       <c r="BE3" s="3" t="n">
         <v>51282</v>
+      </c>
+      <c r="BF3" s="3" t="n">
+        <v>350641</v>
+      </c>
+      <c r="BG3" s="3" t="n">
+        <v>40556</v>
+      </c>
+      <c r="BH3" s="3" t="n">
+        <v>43354</v>
+      </c>
+      <c r="BI3" s="3" t="n">
+        <v>52339</v>
+      </c>
+      <c r="BJ3" s="3" t="n">
+        <v>51522</v>
+      </c>
+      <c r="BK3" s="3" t="n">
+        <v>33904</v>
+      </c>
+      <c r="BL3" s="3" t="n">
+        <v>12676</v>
+      </c>
+      <c r="BM3" s="3" t="n">
+        <v>12494</v>
+      </c>
+      <c r="BN3" s="3" t="n">
+        <v>16061</v>
+      </c>
+      <c r="BO3" s="3" t="n">
+        <v>10856</v>
+      </c>
+      <c r="BP3" s="3" t="n">
+        <v>16450</v>
+      </c>
+      <c r="BQ3" s="3" t="n">
+        <v>29319</v>
+      </c>
+      <c r="BR3" s="3" t="n">
+        <v>31110</v>
       </c>
     </row>
   </sheetData>
@@ -1287,7 +1443,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BE3"/>
+  <dimension ref="A1:BR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1347,6 +1503,19 @@
     <col width="10" customWidth="1" min="55" max="55"/>
     <col width="10" customWidth="1" min="56" max="56"/>
     <col width="10" customWidth="1" min="57" max="57"/>
+    <col width="10" customWidth="1" min="58" max="58"/>
+    <col width="10" customWidth="1" min="59" max="59"/>
+    <col width="10" customWidth="1" min="60" max="60"/>
+    <col width="10" customWidth="1" min="61" max="61"/>
+    <col width="10" customWidth="1" min="62" max="62"/>
+    <col width="10" customWidth="1" min="63" max="63"/>
+    <col width="10" customWidth="1" min="64" max="64"/>
+    <col width="10" customWidth="1" min="65" max="65"/>
+    <col width="10" customWidth="1" min="66" max="66"/>
+    <col width="10" customWidth="1" min="67" max="67"/>
+    <col width="10" customWidth="1" min="68" max="68"/>
+    <col width="10" customWidth="1" min="69" max="69"/>
+    <col width="10" customWidth="1" min="70" max="70"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1633,6 +1802,71 @@
       <c r="BE1" s="1" t="inlineStr">
         <is>
           <t>2021 M12</t>
+        </is>
+      </c>
+      <c r="BF1" s="1" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="BG1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M01</t>
+        </is>
+      </c>
+      <c r="BH1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M02</t>
+        </is>
+      </c>
+      <c r="BI1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M03</t>
+        </is>
+      </c>
+      <c r="BJ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M04</t>
+        </is>
+      </c>
+      <c r="BK1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M05</t>
+        </is>
+      </c>
+      <c r="BL1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M06</t>
+        </is>
+      </c>
+      <c r="BM1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M07</t>
+        </is>
+      </c>
+      <c r="BN1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M08</t>
+        </is>
+      </c>
+      <c r="BO1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M09</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M10</t>
+        </is>
+      </c>
+      <c r="BQ1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M11</t>
+        </is>
+      </c>
+      <c r="BR1" s="1" t="inlineStr">
+        <is>
+          <t>2022 M12</t>
         </is>
       </c>
     </row>
@@ -1766,6 +2000,45 @@
       <c r="BE2" s="3" t="n">
         <v>93</v>
       </c>
+      <c r="BF2" s="3" t="n">
+        <v>1027</v>
+      </c>
+      <c r="BG2" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="BH2" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="BI2" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="BJ2" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="BK2" s="3" t="n">
+        <v>162</v>
+      </c>
+      <c r="BL2" s="3" t="n">
+        <v>136</v>
+      </c>
+      <c r="BM2" s="3" t="n">
+        <v>138</v>
+      </c>
+      <c r="BN2" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="BO2" s="3" t="n">
+        <v>64</v>
+      </c>
+      <c r="BP2" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="BQ2" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="BR2" s="3" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1942,6 +2215,43 @@
       </c>
       <c r="BE3" s="3" t="n">
         <v>279</v>
+      </c>
+      <c r="BF3" s="3" t="n">
+        <v>21041</v>
+      </c>
+      <c r="BG3" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="BH3" s="3" t="n">
+        <v>2626</v>
+      </c>
+      <c r="BI3" s="3" t="n">
+        <v>2592</v>
+      </c>
+      <c r="BJ3" s="2" t="inlineStr"/>
+      <c r="BK3" s="3" t="n">
+        <v>834</v>
+      </c>
+      <c r="BL3" s="3" t="n">
+        <v>1653</v>
+      </c>
+      <c r="BM3" s="3" t="n">
+        <v>2916</v>
+      </c>
+      <c r="BN3" s="3" t="n">
+        <v>1234</v>
+      </c>
+      <c r="BO3" s="3" t="n">
+        <v>1260</v>
+      </c>
+      <c r="BP3" s="3" t="n">
+        <v>4856</v>
+      </c>
+      <c r="BQ3" s="3" t="n">
+        <v>1786</v>
+      </c>
+      <c r="BR3" s="3" t="n">
+        <v>1265</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2023
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2022</v>
+        <v>2023</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>2</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR3"/>
+  <dimension ref="A1:CE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -634,6 +634,19 @@
     <col width="10" customWidth="1" min="68" max="68"/>
     <col width="10" customWidth="1" min="69" max="69"/>
     <col width="10" customWidth="1" min="70" max="70"/>
+    <col width="10" customWidth="1" min="71" max="71"/>
+    <col width="10" customWidth="1" min="72" max="72"/>
+    <col width="10" customWidth="1" min="73" max="73"/>
+    <col width="10" customWidth="1" min="74" max="74"/>
+    <col width="10" customWidth="1" min="75" max="75"/>
+    <col width="10" customWidth="1" min="76" max="76"/>
+    <col width="10" customWidth="1" min="77" max="77"/>
+    <col width="10" customWidth="1" min="78" max="78"/>
+    <col width="10" customWidth="1" min="79" max="79"/>
+    <col width="10" customWidth="1" min="80" max="80"/>
+    <col width="10" customWidth="1" min="81" max="81"/>
+    <col width="10" customWidth="1" min="82" max="82"/>
+    <col width="10" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -987,6 +1000,71 @@
           <t>2022 M12</t>
         </is>
       </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M01</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M02</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M03</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M04</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M05</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M06</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M07</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M08</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M09</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M10</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M11</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1209,6 +1287,45 @@
       <c r="BR2" s="3" t="n">
         <v>28268</v>
       </c>
+      <c r="BS2" s="3" t="n">
+        <v>261115</v>
+      </c>
+      <c r="BT2" s="3" t="n">
+        <v>21512</v>
+      </c>
+      <c r="BU2" s="3" t="n">
+        <v>21302</v>
+      </c>
+      <c r="BV2" s="3" t="n">
+        <v>16891</v>
+      </c>
+      <c r="BW2" s="3" t="n">
+        <v>18037</v>
+      </c>
+      <c r="BX2" s="3" t="n">
+        <v>21503</v>
+      </c>
+      <c r="BY2" s="3" t="n">
+        <v>22078</v>
+      </c>
+      <c r="BZ2" s="3" t="n">
+        <v>26784</v>
+      </c>
+      <c r="CA2" s="3" t="n">
+        <v>14098</v>
+      </c>
+      <c r="CB2" s="3" t="n">
+        <v>27551</v>
+      </c>
+      <c r="CC2" s="3" t="n">
+        <v>25040</v>
+      </c>
+      <c r="CD2" s="3" t="n">
+        <v>20560</v>
+      </c>
+      <c r="CE2" s="3" t="n">
+        <v>25759</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1430,6 +1547,45 @@
       </c>
       <c r="BR3" s="3" t="n">
         <v>31110</v>
+      </c>
+      <c r="BS3" s="3" t="n">
+        <v>354110</v>
+      </c>
+      <c r="BT3" s="3" t="n">
+        <v>24827</v>
+      </c>
+      <c r="BU3" s="3" t="n">
+        <v>23987</v>
+      </c>
+      <c r="BV3" s="3" t="n">
+        <v>25004</v>
+      </c>
+      <c r="BW3" s="3" t="n">
+        <v>26091</v>
+      </c>
+      <c r="BX3" s="3" t="n">
+        <v>21508</v>
+      </c>
+      <c r="BY3" s="3" t="n">
+        <v>30427</v>
+      </c>
+      <c r="BZ3" s="3" t="n">
+        <v>35696</v>
+      </c>
+      <c r="CA3" s="3" t="n">
+        <v>39806</v>
+      </c>
+      <c r="CB3" s="3" t="n">
+        <v>28284</v>
+      </c>
+      <c r="CC3" s="3" t="n">
+        <v>24637</v>
+      </c>
+      <c r="CD3" s="3" t="n">
+        <v>39867</v>
+      </c>
+      <c r="CE3" s="3" t="n">
+        <v>33976</v>
       </c>
     </row>
   </sheetData>
@@ -1443,7 +1599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR3"/>
+  <dimension ref="A1:CE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1516,6 +1672,19 @@
     <col width="10" customWidth="1" min="68" max="68"/>
     <col width="10" customWidth="1" min="69" max="69"/>
     <col width="10" customWidth="1" min="70" max="70"/>
+    <col width="10" customWidth="1" min="71" max="71"/>
+    <col width="10" customWidth="1" min="72" max="72"/>
+    <col width="10" customWidth="1" min="73" max="73"/>
+    <col width="10" customWidth="1" min="74" max="74"/>
+    <col width="10" customWidth="1" min="75" max="75"/>
+    <col width="10" customWidth="1" min="76" max="76"/>
+    <col width="10" customWidth="1" min="77" max="77"/>
+    <col width="10" customWidth="1" min="78" max="78"/>
+    <col width="10" customWidth="1" min="79" max="79"/>
+    <col width="10" customWidth="1" min="80" max="80"/>
+    <col width="10" customWidth="1" min="81" max="81"/>
+    <col width="10" customWidth="1" min="82" max="82"/>
+    <col width="10" customWidth="1" min="83" max="83"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1867,6 +2036,71 @@
       <c r="BR1" s="1" t="inlineStr">
         <is>
           <t>2022 M12</t>
+        </is>
+      </c>
+      <c r="BS1" s="1" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="BT1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M01</t>
+        </is>
+      </c>
+      <c r="BU1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M02</t>
+        </is>
+      </c>
+      <c r="BV1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M03</t>
+        </is>
+      </c>
+      <c r="BW1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M04</t>
+        </is>
+      </c>
+      <c r="BX1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M05</t>
+        </is>
+      </c>
+      <c r="BY1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M06</t>
+        </is>
+      </c>
+      <c r="BZ1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M07</t>
+        </is>
+      </c>
+      <c r="CA1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M08</t>
+        </is>
+      </c>
+      <c r="CB1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M09</t>
+        </is>
+      </c>
+      <c r="CC1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M10</t>
+        </is>
+      </c>
+      <c r="CD1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M11</t>
+        </is>
+      </c>
+      <c r="CE1" s="1" t="inlineStr">
+        <is>
+          <t>2023 M12</t>
         </is>
       </c>
     </row>
@@ -2039,6 +2273,45 @@
       <c r="BR2" s="3" t="n">
         <v>43</v>
       </c>
+      <c r="BS2" s="3" t="n">
+        <v>511</v>
+      </c>
+      <c r="BT2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="BU2" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="BV2" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="BW2" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="BX2" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="BY2" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="BZ2" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="CA2" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="CB2" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="CC2" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="CD2" s="3" t="n">
+        <v>63</v>
+      </c>
+      <c r="CE2" s="3" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2252,6 +2525,45 @@
       </c>
       <c r="BR3" s="3" t="n">
         <v>1265</v>
+      </c>
+      <c r="BS3" s="3" t="n">
+        <v>27696</v>
+      </c>
+      <c r="BT3" s="3" t="n">
+        <v>1288</v>
+      </c>
+      <c r="BU3" s="3" t="n">
+        <v>127</v>
+      </c>
+      <c r="BV3" s="3" t="n">
+        <v>1183</v>
+      </c>
+      <c r="BW3" s="3" t="n">
+        <v>1372</v>
+      </c>
+      <c r="BX3" s="3" t="n">
+        <v>2041</v>
+      </c>
+      <c r="BY3" s="3" t="n">
+        <v>2554</v>
+      </c>
+      <c r="BZ3" s="3" t="n">
+        <v>4806</v>
+      </c>
+      <c r="CA3" s="3" t="n">
+        <v>4707</v>
+      </c>
+      <c r="CB3" s="3" t="n">
+        <v>6185</v>
+      </c>
+      <c r="CC3" s="3" t="n">
+        <v>2811</v>
+      </c>
+      <c r="CD3" s="3" t="n">
+        <v>554</v>
+      </c>
+      <c r="CE3" s="3" t="n">
+        <v>68</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2024
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="D3" s="3" t="n">
         <v>26</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE3"/>
+  <dimension ref="A1:CR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -647,6 +647,19 @@
     <col width="10" customWidth="1" min="81" max="81"/>
     <col width="10" customWidth="1" min="82" max="82"/>
     <col width="10" customWidth="1" min="83" max="83"/>
+    <col width="10" customWidth="1" min="84" max="84"/>
+    <col width="10" customWidth="1" min="85" max="85"/>
+    <col width="10" customWidth="1" min="86" max="86"/>
+    <col width="10" customWidth="1" min="87" max="87"/>
+    <col width="10" customWidth="1" min="88" max="88"/>
+    <col width="10" customWidth="1" min="89" max="89"/>
+    <col width="10" customWidth="1" min="90" max="90"/>
+    <col width="10" customWidth="1" min="91" max="91"/>
+    <col width="10" customWidth="1" min="92" max="92"/>
+    <col width="10" customWidth="1" min="93" max="93"/>
+    <col width="10" customWidth="1" min="94" max="94"/>
+    <col width="10" customWidth="1" min="95" max="95"/>
+    <col width="10" customWidth="1" min="96" max="96"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1065,6 +1078,71 @@
           <t>2023 M12</t>
         </is>
       </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M01</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M02</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M03</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M04</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M05</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M06</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M07</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M08</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M09</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M10</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M11</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1326,6 +1404,45 @@
       <c r="CE2" s="3" t="n">
         <v>25759</v>
       </c>
+      <c r="CF2" s="3" t="n">
+        <v>254952</v>
+      </c>
+      <c r="CG2" s="3" t="n">
+        <v>12855</v>
+      </c>
+      <c r="CH2" s="3" t="n">
+        <v>16323</v>
+      </c>
+      <c r="CI2" s="3" t="n">
+        <v>17948</v>
+      </c>
+      <c r="CJ2" s="3" t="n">
+        <v>22821</v>
+      </c>
+      <c r="CK2" s="3" t="n">
+        <v>21050</v>
+      </c>
+      <c r="CL2" s="3" t="n">
+        <v>23391</v>
+      </c>
+      <c r="CM2" s="3" t="n">
+        <v>24212</v>
+      </c>
+      <c r="CN2" s="3" t="n">
+        <v>24312</v>
+      </c>
+      <c r="CO2" s="3" t="n">
+        <v>20039</v>
+      </c>
+      <c r="CP2" s="3" t="n">
+        <v>25493</v>
+      </c>
+      <c r="CQ2" s="3" t="n">
+        <v>25232</v>
+      </c>
+      <c r="CR2" s="3" t="n">
+        <v>21276</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1586,6 +1703,45 @@
       </c>
       <c r="CE3" s="3" t="n">
         <v>33976</v>
+      </c>
+      <c r="CF3" s="3" t="n">
+        <v>369820</v>
+      </c>
+      <c r="CG3" s="3" t="n">
+        <v>33333</v>
+      </c>
+      <c r="CH3" s="3" t="n">
+        <v>25527</v>
+      </c>
+      <c r="CI3" s="3" t="n">
+        <v>23836</v>
+      </c>
+      <c r="CJ3" s="3" t="n">
+        <v>26483</v>
+      </c>
+      <c r="CK3" s="3" t="n">
+        <v>30474</v>
+      </c>
+      <c r="CL3" s="3" t="n">
+        <v>31887</v>
+      </c>
+      <c r="CM3" s="3" t="n">
+        <v>32270</v>
+      </c>
+      <c r="CN3" s="3" t="n">
+        <v>29464</v>
+      </c>
+      <c r="CO3" s="3" t="n">
+        <v>19004</v>
+      </c>
+      <c r="CP3" s="3" t="n">
+        <v>31421</v>
+      </c>
+      <c r="CQ3" s="3" t="n">
+        <v>44030</v>
+      </c>
+      <c r="CR3" s="3" t="n">
+        <v>42091</v>
       </c>
     </row>
   </sheetData>
@@ -1599,7 +1755,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CE3"/>
+  <dimension ref="A1:CR3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1685,6 +1841,19 @@
     <col width="10" customWidth="1" min="81" max="81"/>
     <col width="10" customWidth="1" min="82" max="82"/>
     <col width="10" customWidth="1" min="83" max="83"/>
+    <col width="10" customWidth="1" min="84" max="84"/>
+    <col width="10" customWidth="1" min="85" max="85"/>
+    <col width="10" customWidth="1" min="86" max="86"/>
+    <col width="10" customWidth="1" min="87" max="87"/>
+    <col width="10" customWidth="1" min="88" max="88"/>
+    <col width="10" customWidth="1" min="89" max="89"/>
+    <col width="10" customWidth="1" min="90" max="90"/>
+    <col width="10" customWidth="1" min="91" max="91"/>
+    <col width="10" customWidth="1" min="92" max="92"/>
+    <col width="10" customWidth="1" min="93" max="93"/>
+    <col width="10" customWidth="1" min="94" max="94"/>
+    <col width="10" customWidth="1" min="95" max="95"/>
+    <col width="10" customWidth="1" min="96" max="96"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2101,6 +2270,71 @@
       <c r="CE1" s="1" t="inlineStr">
         <is>
           <t>2023 M12</t>
+        </is>
+      </c>
+      <c r="CF1" s="1" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CG1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M01</t>
+        </is>
+      </c>
+      <c r="CH1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M02</t>
+        </is>
+      </c>
+      <c r="CI1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M03</t>
+        </is>
+      </c>
+      <c r="CJ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M04</t>
+        </is>
+      </c>
+      <c r="CK1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M05</t>
+        </is>
+      </c>
+      <c r="CL1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M06</t>
+        </is>
+      </c>
+      <c r="CM1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M07</t>
+        </is>
+      </c>
+      <c r="CN1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M08</t>
+        </is>
+      </c>
+      <c r="CO1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M09</t>
+        </is>
+      </c>
+      <c r="CP1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M10</t>
+        </is>
+      </c>
+      <c r="CQ1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M11</t>
+        </is>
+      </c>
+      <c r="CR1" s="1" t="inlineStr">
+        <is>
+          <t>2024 M12</t>
         </is>
       </c>
     </row>
@@ -2312,6 +2546,45 @@
       <c r="CE2" s="3" t="n">
         <v>60</v>
       </c>
+      <c r="CF2" s="3" t="n">
+        <v>157</v>
+      </c>
+      <c r="CG2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="CH2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="CI2" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="CJ2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="CK2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="CL2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="CM2" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="CN2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="CO2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="CP2" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="CQ2" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="CR2" s="3" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2564,6 +2837,45 @@
       </c>
       <c r="CE3" s="3" t="n">
         <v>68</v>
+      </c>
+      <c r="CF3" s="3" t="n">
+        <v>3471</v>
+      </c>
+      <c r="CG3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="CH3" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="CI3" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="CJ3" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="CK3" s="3" t="n">
+        <v>1220</v>
+      </c>
+      <c r="CL3" s="3" t="n">
+        <v>1344</v>
+      </c>
+      <c r="CM3" s="3" t="n">
+        <v>297</v>
+      </c>
+      <c r="CN3" s="3" t="n">
+        <v>248</v>
+      </c>
+      <c r="CO3" s="3" t="n">
+        <v>134</v>
+      </c>
+      <c r="CP3" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="CQ3" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="CR3" s="3" t="n">
+        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2025
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D2" s="3" t="n">
         <v>26</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>2</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR3"/>
+  <dimension ref="A1:DE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -660,6 +660,19 @@
     <col width="10" customWidth="1" min="94" max="94"/>
     <col width="10" customWidth="1" min="95" max="95"/>
     <col width="10" customWidth="1" min="96" max="96"/>
+    <col width="10" customWidth="1" min="97" max="97"/>
+    <col width="10" customWidth="1" min="98" max="98"/>
+    <col width="10" customWidth="1" min="99" max="99"/>
+    <col width="10" customWidth="1" min="100" max="100"/>
+    <col width="10" customWidth="1" min="101" max="101"/>
+    <col width="10" customWidth="1" min="102" max="102"/>
+    <col width="10" customWidth="1" min="103" max="103"/>
+    <col width="10" customWidth="1" min="104" max="104"/>
+    <col width="10" customWidth="1" min="105" max="105"/>
+    <col width="10" customWidth="1" min="106" max="106"/>
+    <col width="10" customWidth="1" min="107" max="107"/>
+    <col width="10" customWidth="1" min="108" max="108"/>
+    <col width="10" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1143,6 +1156,71 @@
           <t>2024 M12</t>
         </is>
       </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M01</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M02</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M03</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M04</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M05</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M06</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M07</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M08</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M09</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M10</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M11</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M12</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1443,6 +1521,45 @@
       <c r="CR2" s="3" t="n">
         <v>21276</v>
       </c>
+      <c r="CS2" s="3" t="n">
+        <v>332087</v>
+      </c>
+      <c r="CT2" s="3" t="n">
+        <v>31962</v>
+      </c>
+      <c r="CU2" s="3" t="n">
+        <v>17366</v>
+      </c>
+      <c r="CV2" s="3" t="n">
+        <v>31866</v>
+      </c>
+      <c r="CW2" s="3" t="n">
+        <v>24700</v>
+      </c>
+      <c r="CX2" s="3" t="n">
+        <v>28087</v>
+      </c>
+      <c r="CY2" s="3" t="n">
+        <v>26105</v>
+      </c>
+      <c r="CZ2" s="3" t="n">
+        <v>26014</v>
+      </c>
+      <c r="DA2" s="3" t="n">
+        <v>30369</v>
+      </c>
+      <c r="DB2" s="3" t="n">
+        <v>28304</v>
+      </c>
+      <c r="DC2" s="3" t="n">
+        <v>28793</v>
+      </c>
+      <c r="DD2" s="3" t="n">
+        <v>31682</v>
+      </c>
+      <c r="DE2" s="3" t="n">
+        <v>26839</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1742,6 +1859,45 @@
       </c>
       <c r="CR3" s="3" t="n">
         <v>42091</v>
+      </c>
+      <c r="CS3" s="3" t="n">
+        <v>436554</v>
+      </c>
+      <c r="CT3" s="3" t="n">
+        <v>29462</v>
+      </c>
+      <c r="CU3" s="3" t="n">
+        <v>35826</v>
+      </c>
+      <c r="CV3" s="3" t="n">
+        <v>27499</v>
+      </c>
+      <c r="CW3" s="3" t="n">
+        <v>24235</v>
+      </c>
+      <c r="CX3" s="3" t="n">
+        <v>33609</v>
+      </c>
+      <c r="CY3" s="3" t="n">
+        <v>33331</v>
+      </c>
+      <c r="CZ3" s="3" t="n">
+        <v>36627</v>
+      </c>
+      <c r="DA3" s="3" t="n">
+        <v>34830</v>
+      </c>
+      <c r="DB3" s="3" t="n">
+        <v>37664</v>
+      </c>
+      <c r="DC3" s="3" t="n">
+        <v>42377</v>
+      </c>
+      <c r="DD3" s="3" t="n">
+        <v>44953</v>
+      </c>
+      <c r="DE3" s="3" t="n">
+        <v>56141</v>
       </c>
     </row>
   </sheetData>
@@ -1755,7 +1911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:CR3"/>
+  <dimension ref="A1:DE3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -1854,6 +2010,19 @@
     <col width="10" customWidth="1" min="94" max="94"/>
     <col width="10" customWidth="1" min="95" max="95"/>
     <col width="10" customWidth="1" min="96" max="96"/>
+    <col width="10" customWidth="1" min="97" max="97"/>
+    <col width="10" customWidth="1" min="98" max="98"/>
+    <col width="10" customWidth="1" min="99" max="99"/>
+    <col width="10" customWidth="1" min="100" max="100"/>
+    <col width="10" customWidth="1" min="101" max="101"/>
+    <col width="10" customWidth="1" min="102" max="102"/>
+    <col width="10" customWidth="1" min="103" max="103"/>
+    <col width="10" customWidth="1" min="104" max="104"/>
+    <col width="10" customWidth="1" min="105" max="105"/>
+    <col width="10" customWidth="1" min="106" max="106"/>
+    <col width="10" customWidth="1" min="107" max="107"/>
+    <col width="10" customWidth="1" min="108" max="108"/>
+    <col width="10" customWidth="1" min="109" max="109"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2335,6 +2504,71 @@
       <c r="CR1" s="1" t="inlineStr">
         <is>
           <t>2024 M12</t>
+        </is>
+      </c>
+      <c r="CS1" s="1" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="CT1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M01</t>
+        </is>
+      </c>
+      <c r="CU1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M02</t>
+        </is>
+      </c>
+      <c r="CV1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M03</t>
+        </is>
+      </c>
+      <c r="CW1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M04</t>
+        </is>
+      </c>
+      <c r="CX1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M05</t>
+        </is>
+      </c>
+      <c r="CY1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M06</t>
+        </is>
+      </c>
+      <c r="CZ1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M07</t>
+        </is>
+      </c>
+      <c r="DA1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M08</t>
+        </is>
+      </c>
+      <c r="DB1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M09</t>
+        </is>
+      </c>
+      <c r="DC1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M10</t>
+        </is>
+      </c>
+      <c r="DD1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M11</t>
+        </is>
+      </c>
+      <c r="DE1" s="1" t="inlineStr">
+        <is>
+          <t>2025 M12</t>
         </is>
       </c>
     </row>
@@ -2585,6 +2819,45 @@
       <c r="CR2" s="3" t="n">
         <v>10</v>
       </c>
+      <c r="CS2" s="3" t="n">
+        <v>144</v>
+      </c>
+      <c r="CT2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="CU2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="CV2" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="CW2" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="CX2" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="CY2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="CZ2" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="DA2" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="DB2" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="DC2" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="DD2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="DE2" s="3" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -2876,6 +3149,43 @@
       </c>
       <c r="CR3" s="3" t="n">
         <v>37</v>
+      </c>
+      <c r="CS3" s="3" t="n">
+        <v>77041</v>
+      </c>
+      <c r="CT3" s="2" t="inlineStr"/>
+      <c r="CU3" s="3" t="n">
+        <v>2478</v>
+      </c>
+      <c r="CV3" s="3" t="n">
+        <v>574</v>
+      </c>
+      <c r="CW3" s="3" t="n">
+        <v>4197</v>
+      </c>
+      <c r="CX3" s="3" t="n">
+        <v>6824</v>
+      </c>
+      <c r="CY3" s="3" t="n">
+        <v>6383</v>
+      </c>
+      <c r="CZ3" s="3" t="n">
+        <v>10332</v>
+      </c>
+      <c r="DA3" s="3" t="n">
+        <v>8925</v>
+      </c>
+      <c r="DB3" s="3" t="n">
+        <v>11801</v>
+      </c>
+      <c r="DC3" s="3" t="n">
+        <v>8664</v>
+      </c>
+      <c r="DD3" s="3" t="n">
+        <v>8549</v>
+      </c>
+      <c r="DE3" s="3" t="n">
+        <v>8314</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Append GUS gas data for 2026
</commit_message>
<xml_diff>
--- a/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
+++ b/gus_dbw_trade/gus_gas_TJ_2018_plus_IMPORT_EXPORT_MASTER.xlsx
@@ -508,10 +508,10 @@
         </is>
       </c>
       <c r="C2" s="3" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D2" s="3" t="n">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E2" s="3" t="n">
         <v>2</v>
@@ -535,10 +535,10 @@
         </is>
       </c>
       <c r="C3" s="3" t="n">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D3" s="3" t="n">
-        <v>25</v>
+        <v>6</v>
       </c>
       <c r="E3" s="3" t="n">
         <v>2</v>
@@ -561,7 +561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE3"/>
+  <dimension ref="A1:DH3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37" customWidth="1" min="1" max="1"/>
@@ -673,6 +673,9 @@
     <col width="10" customWidth="1" min="107" max="107"/>
     <col width="10" customWidth="1" min="108" max="108"/>
     <col width="10" customWidth="1" min="109" max="109"/>
+    <col width="10" customWidth="1" min="110" max="110"/>
+    <col width="10" customWidth="1" min="111" max="111"/>
+    <col width="10" customWidth="1" min="112" max="112"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1221,6 +1224,21 @@
           <t>2025 M12</t>
         </is>
       </c>
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>2026 M01</t>
+        </is>
+      </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>2026 M02</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr">
+        <is>
+          <t>2026 M03</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -1560,6 +1578,15 @@
       <c r="DE2" s="3" t="n">
         <v>26839</v>
       </c>
+      <c r="DF2" s="3" t="n">
+        <v>33129</v>
+      </c>
+      <c r="DG2" s="3" t="n">
+        <v>29470</v>
+      </c>
+      <c r="DH2" s="3" t="n">
+        <v>30576</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -1898,6 +1925,15 @@
       </c>
       <c r="DE3" s="3" t="n">
         <v>56141</v>
+      </c>
+      <c r="DF3" s="3" t="n">
+        <v>62191</v>
+      </c>
+      <c r="DG3" s="3" t="n">
+        <v>58555</v>
+      </c>
+      <c r="DH3" s="3" t="n">
+        <v>36685</v>
       </c>
     </row>
   </sheetData>
@@ -1911,7 +1947,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DE3"/>
+  <dimension ref="A1:DH3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -2023,6 +2059,9 @@
     <col width="10" customWidth="1" min="107" max="107"/>
     <col width="10" customWidth="1" min="108" max="108"/>
     <col width="10" customWidth="1" min="109" max="109"/>
+    <col width="10" customWidth="1" min="110" max="110"/>
+    <col width="10" customWidth="1" min="111" max="111"/>
+    <col width="10" customWidth="1" min="112" max="112"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2569,6 +2608,21 @@
       <c r="DE1" s="1" t="inlineStr">
         <is>
           <t>2025 M12</t>
+        </is>
+      </c>
+      <c r="DF1" s="1" t="inlineStr">
+        <is>
+          <t>2026 M01</t>
+        </is>
+      </c>
+      <c r="DG1" s="1" t="inlineStr">
+        <is>
+          <t>2026 M02</t>
+        </is>
+      </c>
+      <c r="DH1" s="1" t="inlineStr">
+        <is>
+          <t>2026 M03</t>
         </is>
       </c>
     </row>
@@ -2858,6 +2912,15 @@
       <c r="DE2" s="3" t="n">
         <v>6</v>
       </c>
+      <c r="DF2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="DG2" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="DH2" s="3" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -3186,6 +3249,15 @@
       </c>
       <c r="DE3" s="3" t="n">
         <v>8314</v>
+      </c>
+      <c r="DF3" s="3" t="n">
+        <v>8751</v>
+      </c>
+      <c r="DG3" s="3" t="n">
+        <v>10064</v>
+      </c>
+      <c r="DH3" s="3" t="n">
+        <v>7151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>